<commit_message>
Update on nn regressor and decision tree
</commit_message>
<xml_diff>
--- a/regression_deneme/regression_with_nn/Mürselpaşa Bulvarı_monthly_true_and_predicted_test.xlsx
+++ b/regression_deneme/regression_with_nn/Mürselpaşa Bulvarı_monthly_true_and_predicted_test.xlsx
@@ -461,7 +461,7 @@
         <v>76</v>
       </c>
       <c r="D2" t="n">
-        <v>70.61810482711518</v>
+        <v>70.21083138677764</v>
       </c>
     </row>
     <row r="3">
@@ -475,7 +475,7 @@
         <v>46</v>
       </c>
       <c r="D3" t="n">
-        <v>55.2614546180779</v>
+        <v>50.98598129893345</v>
       </c>
     </row>
     <row r="4">
@@ -489,7 +489,7 @@
         <v>44</v>
       </c>
       <c r="D4" t="n">
-        <v>43.69706642459774</v>
+        <v>47.06855843769061</v>
       </c>
     </row>
     <row r="5">
@@ -503,7 +503,7 @@
         <v>56</v>
       </c>
       <c r="D5" t="n">
-        <v>52.73696974955777</v>
+        <v>52.24407942223753</v>
       </c>
     </row>
     <row r="6">
@@ -517,7 +517,7 @@
         <v>42</v>
       </c>
       <c r="D6" t="n">
-        <v>48.73049457877583</v>
+        <v>45.23764215855926</v>
       </c>
     </row>
     <row r="7">
@@ -531,7 +531,7 @@
         <v>44</v>
       </c>
       <c r="D7" t="n">
-        <v>44.13801380169159</v>
+        <v>45.47102468626358</v>
       </c>
     </row>
     <row r="8">
@@ -545,7 +545,7 @@
         <v>45</v>
       </c>
       <c r="D8" t="n">
-        <v>44.22948975531114</v>
+        <v>44.95218154286693</v>
       </c>
     </row>
   </sheetData>

</xml_diff>